<commit_message>
fix: resolve pipeline failures in security review and load tests
</commit_message>
<xml_diff>
--- a/load-tests/load-test-report.xlsx
+++ b/load-tests/load-test-report.xlsx
@@ -47,7 +47,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -64,12 +64,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="002F5496"/>
         <bgColor rgb="002F5496"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-        <bgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -100,7 +94,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -215,12 +209,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'RPS Timeline'!$A$2:$A$62</f>
+              <f>'RPS Timeline'!$A$2:$A$7</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'RPS Timeline'!$B$2:$B$62</f>
+              <f>'RPS Timeline'!$B$2:$B$7</f>
             </numRef>
           </val>
         </ser>
@@ -650,7 +644,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>60</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
@@ -671,7 +665,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-09-02T09:09:49.075029</t>
+          <t>2026-09-02T10:40:13.193295</t>
         </is>
       </c>
     </row>
@@ -694,7 +688,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>24566</v>
+        <v>750</v>
       </c>
     </row>
     <row r="11">
@@ -704,7 +698,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>12404.45</v>
+        <v>379.95</v>
       </c>
     </row>
     <row r="12">
@@ -714,7 +708,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>409.41</v>
+        <v>149.88</v>
       </c>
     </row>
     <row r="13">
@@ -724,7 +718,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>619</v>
+        <v>179</v>
       </c>
     </row>
     <row r="14">
@@ -734,7 +728,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>102</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
@@ -756,7 +750,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>244.62</v>
+        <v>33.42</v>
       </c>
     </row>
     <row r="18">
@@ -766,7 +760,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>73.56999999999999</v>
+        <v>10.81</v>
       </c>
     </row>
     <row r="19">
@@ -776,7 +770,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1052.27</v>
+        <v>323.53</v>
       </c>
     </row>
     <row r="20">
@@ -786,7 +780,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>207.02</v>
+        <v>27.46</v>
       </c>
     </row>
     <row r="21">
@@ -796,7 +790,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>406.84</v>
+        <v>51.9</v>
       </c>
     </row>
     <row r="22">
@@ -806,7 +800,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>468.78</v>
+        <v>59.48</v>
       </c>
     </row>
     <row r="23">
@@ -816,7 +810,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>720.17</v>
+        <v>83.97</v>
       </c>
     </row>
     <row r="24">
@@ -826,7 +820,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>124.92</v>
+        <v>27.66</v>
       </c>
     </row>
     <row r="25">
@@ -848,7 +842,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>24566</v>
+        <v>750</v>
       </c>
     </row>
     <row r="28">
@@ -890,7 +884,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>22092</v>
+        <v>675</v>
       </c>
     </row>
     <row r="33">
@@ -900,7 +894,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>2474</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -986,25 +980,25 @@
         </is>
       </c>
       <c r="B2" s="5" t="n">
-        <v>2500</v>
+        <v>75</v>
       </c>
       <c r="C2" s="6" t="n">
-        <v>430.02</v>
+        <v>51.83</v>
       </c>
       <c r="D2" s="5" t="n">
-        <v>311.23</v>
+        <v>35.22</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>831.48</v>
+        <v>86.95999999999999</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>389.66</v>
+        <v>50.04</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>749.6799999999999</v>
+        <v>71.98</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>802.87</v>
+        <v>86.95999999999999</v>
       </c>
       <c r="I2" s="5" t="n">
         <v>0</v>
@@ -1013,29 +1007,29 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Get Security Questions</t>
+          <t>Health Check</t>
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>2500</v>
+        <v>76</v>
       </c>
       <c r="C3" s="6" t="n">
-        <v>360.02</v>
+        <v>45.22</v>
       </c>
       <c r="D3" s="5" t="n">
-        <v>180.01</v>
+        <v>13.18</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>764.08</v>
+        <v>323.53</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>345.64</v>
+        <v>25.03</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>482.86</v>
+        <v>322.32</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>677.24</v>
+        <v>323.53</v>
       </c>
       <c r="I3" s="5" t="n">
         <v>0</v>
@@ -1048,25 +1042,25 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>2474</v>
+        <v>75</v>
       </c>
       <c r="C4" s="6" t="n">
-        <v>341.6</v>
+        <v>43.94</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>217.75</v>
+        <v>25.09</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>1052.27</v>
+        <v>83.97</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>307.34</v>
+        <v>42.36</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>494.64</v>
+        <v>68.36</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>707.49</v>
+        <v>83.97</v>
       </c>
       <c r="I4" s="5" t="n">
         <v>0</v>
@@ -1075,29 +1069,29 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Marketplace Catalog</t>
+          <t>Get Security Questions</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>2407</v>
+        <v>76</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>233.86</v>
+        <v>43.42</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>128.55</v>
+        <v>20.68</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>869.72</v>
+        <v>106.26</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>205.5</v>
+        <v>42.74</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>345.72</v>
+        <v>63.23</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>743.72</v>
+        <v>106.26</v>
       </c>
       <c r="I5" s="5" t="n">
         <v>0</v>
@@ -1106,29 +1100,29 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Marketplace Models</t>
+          <t>Marketplace Catalog</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>2402</v>
+        <v>74</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>229.64</v>
+        <v>31.55</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>136.4</v>
+        <v>15.31</v>
       </c>
       <c r="E6" s="5" t="n">
-        <v>877</v>
+        <v>66.36</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>208.39</v>
+        <v>27.81</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>322.33</v>
+        <v>53.84</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>464.65</v>
+        <v>66.36</v>
       </c>
       <c r="I6" s="5" t="n">
         <v>0</v>
@@ -1137,29 +1131,29 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Health Check</t>
+          <t>Marketplace Models</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>2500</v>
+        <v>73</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>220.19</v>
+        <v>30.87</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>119.67</v>
+        <v>15.11</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>865.58</v>
+        <v>65.25</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>201.87</v>
+        <v>28.5</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>373.69</v>
+        <v>57.13</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>454.56</v>
+        <v>65.25</v>
       </c>
       <c r="I7" s="5" t="n">
         <v>0</v>
@@ -1168,29 +1162,29 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Root / SPA</t>
+          <t>Pre-Registration TOTP</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>2500</v>
+        <v>75</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>194.04</v>
+        <v>26.99</v>
       </c>
       <c r="D8" s="5" t="n">
-        <v>88.62</v>
+        <v>15.87</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>540.58</v>
+        <v>58.09</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>178.07</v>
+        <v>25.78</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>310.1</v>
+        <v>37.53</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>358.89</v>
+        <v>58.09</v>
       </c>
       <c r="I8" s="5" t="n">
         <v>0</v>
@@ -1199,29 +1193,29 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Compliance Frameworks</t>
+          <t>Root / SPA</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>2415</v>
+        <v>76</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>148.13</v>
+        <v>22.38</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>73.56999999999999</v>
+        <v>11.91</v>
       </c>
       <c r="E9" s="5" t="n">
-        <v>853.59</v>
+        <v>49.53</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>128.94</v>
+        <v>21.75</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>210.89</v>
+        <v>31.37</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>599.33</v>
+        <v>49.53</v>
       </c>
       <c r="I9" s="5" t="n">
         <v>0</v>
@@ -1234,25 +1228,25 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>2427</v>
+        <v>75</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>141.91</v>
+        <v>19.29</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>75.93000000000001</v>
+        <v>11.42</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>838.16</v>
+        <v>44.64</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>123.88</v>
+        <v>17.04</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>197.08</v>
+        <v>39.44</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>632.01</v>
+        <v>44.64</v>
       </c>
       <c r="I10" s="5" t="n">
         <v>0</v>
@@ -1261,29 +1255,29 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Pre-Registration TOTP</t>
+          <t>Compliance Frameworks</t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>2441</v>
+        <v>75</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>138.01</v>
+        <v>18.52</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>81.89</v>
+        <v>10.81</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>873.8</v>
+        <v>45.58</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>122.87</v>
+        <v>18.12</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>202.22</v>
+        <v>25.02</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>438.32</v>
+        <v>45.58</v>
       </c>
       <c r="I11" s="5" t="n">
         <v>0</v>
@@ -1301,7 +1295,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C62"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1331,10 +1325,10 @@
         <v>0</v>
       </c>
       <c r="B2" t="n">
-        <v>282</v>
+        <v>94</v>
       </c>
       <c r="C2" t="n">
-        <v>282</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3">
@@ -1342,10 +1336,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="n">
-        <v>472</v>
+        <v>167</v>
       </c>
       <c r="C3" t="n">
-        <v>754</v>
+        <v>261</v>
       </c>
     </row>
     <row r="4">
@@ -1353,10 +1347,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="n">
-        <v>501</v>
+        <v>143</v>
       </c>
       <c r="C4" t="n">
-        <v>1255</v>
+        <v>404</v>
       </c>
     </row>
     <row r="5">
@@ -1364,10 +1358,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="n">
-        <v>552</v>
+        <v>162</v>
       </c>
       <c r="C5" t="n">
-        <v>1807</v>
+        <v>566</v>
       </c>
     </row>
     <row r="6">
@@ -1375,10 +1369,10 @@
         <v>4</v>
       </c>
       <c r="B6" t="n">
-        <v>442</v>
+        <v>179</v>
       </c>
       <c r="C6" t="n">
-        <v>2249</v>
+        <v>745</v>
       </c>
     </row>
     <row r="7">
@@ -1386,615 +1380,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="n">
-        <v>517</v>
+        <v>5</v>
       </c>
       <c r="C7" t="n">
-        <v>2766</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>6</v>
-      </c>
-      <c r="B8" t="n">
-        <v>514</v>
-      </c>
-      <c r="C8" t="n">
-        <v>3280</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>7</v>
-      </c>
-      <c r="B9" t="n">
-        <v>550</v>
-      </c>
-      <c r="C9" t="n">
-        <v>3830</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>8</v>
-      </c>
-      <c r="B10" t="n">
-        <v>428</v>
-      </c>
-      <c r="C10" t="n">
-        <v>4258</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>9</v>
-      </c>
-      <c r="B11" t="n">
-        <v>522</v>
-      </c>
-      <c r="C11" t="n">
-        <v>4780</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>10</v>
-      </c>
-      <c r="B12" t="n">
-        <v>446</v>
-      </c>
-      <c r="C12" t="n">
-        <v>5226</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>11</v>
-      </c>
-      <c r="B13" t="n">
-        <v>389</v>
-      </c>
-      <c r="C13" t="n">
-        <v>5615</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>12</v>
-      </c>
-      <c r="B14" t="n">
-        <v>499</v>
-      </c>
-      <c r="C14" t="n">
-        <v>6114</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>13</v>
-      </c>
-      <c r="B15" t="n">
-        <v>348</v>
-      </c>
-      <c r="C15" t="n">
-        <v>6462</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>14</v>
-      </c>
-      <c r="B16" t="n">
-        <v>619</v>
-      </c>
-      <c r="C16" t="n">
-        <v>7081</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>15</v>
-      </c>
-      <c r="B17" t="n">
-        <v>386</v>
-      </c>
-      <c r="C17" t="n">
-        <v>7467</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>16</v>
-      </c>
-      <c r="B18" t="n">
-        <v>573</v>
-      </c>
-      <c r="C18" t="n">
-        <v>8040</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>17</v>
-      </c>
-      <c r="B19" t="n">
-        <v>332</v>
-      </c>
-      <c r="C19" t="n">
-        <v>8372</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>18</v>
-      </c>
-      <c r="B20" t="n">
-        <v>608</v>
-      </c>
-      <c r="C20" t="n">
-        <v>8980</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>19</v>
-      </c>
-      <c r="B21" t="n">
-        <v>373</v>
-      </c>
-      <c r="C21" t="n">
-        <v>9353</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>20</v>
-      </c>
-      <c r="B22" t="n">
-        <v>581</v>
-      </c>
-      <c r="C22" t="n">
-        <v>9934</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>21</v>
-      </c>
-      <c r="B23" t="n">
-        <v>417</v>
-      </c>
-      <c r="C23" t="n">
-        <v>10351</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>22</v>
-      </c>
-      <c r="B24" t="n">
-        <v>574</v>
-      </c>
-      <c r="C24" t="n">
-        <v>10925</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>23</v>
-      </c>
-      <c r="B25" t="n">
-        <v>362</v>
-      </c>
-      <c r="C25" t="n">
-        <v>11287</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>24</v>
-      </c>
-      <c r="B26" t="n">
-        <v>518</v>
-      </c>
-      <c r="C26" t="n">
-        <v>11805</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>25</v>
-      </c>
-      <c r="B27" t="n">
-        <v>480</v>
-      </c>
-      <c r="C27" t="n">
-        <v>12285</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>26</v>
-      </c>
-      <c r="B28" t="n">
-        <v>501</v>
-      </c>
-      <c r="C28" t="n">
-        <v>12786</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>27</v>
-      </c>
-      <c r="B29" t="n">
-        <v>494</v>
-      </c>
-      <c r="C29" t="n">
-        <v>13280</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>28</v>
-      </c>
-      <c r="B30" t="n">
-        <v>514</v>
-      </c>
-      <c r="C30" t="n">
-        <v>13794</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>29</v>
-      </c>
-      <c r="B31" t="n">
-        <v>464</v>
-      </c>
-      <c r="C31" t="n">
-        <v>14258</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>30</v>
-      </c>
-      <c r="B32" t="n">
-        <v>490</v>
-      </c>
-      <c r="C32" t="n">
-        <v>14748</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>31</v>
-      </c>
-      <c r="B33" t="n">
-        <v>509</v>
-      </c>
-      <c r="C33" t="n">
-        <v>15257</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="n">
-        <v>32</v>
-      </c>
-      <c r="B34" t="n">
-        <v>418</v>
-      </c>
-      <c r="C34" t="n">
-        <v>15675</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="n">
-        <v>33</v>
-      </c>
-      <c r="B35" t="n">
-        <v>352</v>
-      </c>
-      <c r="C35" t="n">
-        <v>16027</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
-        <v>34</v>
-      </c>
-      <c r="B36" t="n">
-        <v>297</v>
-      </c>
-      <c r="C36" t="n">
-        <v>16324</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="n">
-        <v>35</v>
-      </c>
-      <c r="B37" t="n">
-        <v>419</v>
-      </c>
-      <c r="C37" t="n">
-        <v>16743</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="n">
-        <v>36</v>
-      </c>
-      <c r="B38" t="n">
-        <v>427</v>
-      </c>
-      <c r="C38" t="n">
-        <v>17170</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="n">
-        <v>37</v>
-      </c>
-      <c r="B39" t="n">
-        <v>148</v>
-      </c>
-      <c r="C39" t="n">
-        <v>17318</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="n">
-        <v>38</v>
-      </c>
-      <c r="B40" t="n">
-        <v>340</v>
-      </c>
-      <c r="C40" t="n">
-        <v>17658</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="n">
-        <v>39</v>
-      </c>
-      <c r="B41" t="n">
-        <v>117</v>
-      </c>
-      <c r="C41" t="n">
-        <v>17775</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="n">
-        <v>40</v>
-      </c>
-      <c r="B42" t="n">
-        <v>325</v>
-      </c>
-      <c r="C42" t="n">
-        <v>18100</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
-        <v>41</v>
-      </c>
-      <c r="B43" t="n">
-        <v>276</v>
-      </c>
-      <c r="C43" t="n">
-        <v>18376</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="n">
-        <v>42</v>
-      </c>
-      <c r="B44" t="n">
-        <v>394</v>
-      </c>
-      <c r="C44" t="n">
-        <v>18770</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="n">
-        <v>43</v>
-      </c>
-      <c r="B45" t="n">
-        <v>400</v>
-      </c>
-      <c r="C45" t="n">
-        <v>19170</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="n">
-        <v>44</v>
-      </c>
-      <c r="B46" t="n">
-        <v>274</v>
-      </c>
-      <c r="C46" t="n">
-        <v>19444</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="n">
-        <v>45</v>
-      </c>
-      <c r="B47" t="n">
-        <v>409</v>
-      </c>
-      <c r="C47" t="n">
-        <v>19853</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="n">
-        <v>46</v>
-      </c>
-      <c r="B48" t="n">
-        <v>345</v>
-      </c>
-      <c r="C48" t="n">
-        <v>20198</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="n">
-        <v>47</v>
-      </c>
-      <c r="B49" t="n">
-        <v>190</v>
-      </c>
-      <c r="C49" t="n">
-        <v>20388</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="n">
-        <v>48</v>
-      </c>
-      <c r="B50" t="n">
-        <v>404</v>
-      </c>
-      <c r="C50" t="n">
-        <v>20792</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="n">
-        <v>49</v>
-      </c>
-      <c r="B51" t="n">
-        <v>356</v>
-      </c>
-      <c r="C51" t="n">
-        <v>21148</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="n">
-        <v>50</v>
-      </c>
-      <c r="B52" t="n">
-        <v>285</v>
-      </c>
-      <c r="C52" t="n">
-        <v>21433</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="n">
-        <v>51</v>
-      </c>
-      <c r="B53" t="n">
-        <v>417</v>
-      </c>
-      <c r="C53" t="n">
-        <v>21850</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="n">
-        <v>52</v>
-      </c>
-      <c r="B54" t="n">
-        <v>349</v>
-      </c>
-      <c r="C54" t="n">
-        <v>22199</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="n">
-        <v>53</v>
-      </c>
-      <c r="B55" t="n">
-        <v>299</v>
-      </c>
-      <c r="C55" t="n">
-        <v>22498</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="n">
-        <v>54</v>
-      </c>
-      <c r="B56" t="n">
-        <v>384</v>
-      </c>
-      <c r="C56" t="n">
-        <v>22882</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="n">
-        <v>55</v>
-      </c>
-      <c r="B57" t="n">
-        <v>349</v>
-      </c>
-      <c r="C57" t="n">
-        <v>23231</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="n">
-        <v>56</v>
-      </c>
-      <c r="B58" t="n">
-        <v>231</v>
-      </c>
-      <c r="C58" t="n">
-        <v>23462</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="n">
-        <v>57</v>
-      </c>
-      <c r="B59" t="n">
-        <v>356</v>
-      </c>
-      <c r="C59" t="n">
-        <v>23818</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="n">
-        <v>58</v>
-      </c>
-      <c r="B60" t="n">
-        <v>346</v>
-      </c>
-      <c r="C60" t="n">
-        <v>24164</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="n">
-        <v>59</v>
-      </c>
-      <c r="B61" t="n">
-        <v>300</v>
-      </c>
-      <c r="C61" t="n">
-        <v>24464</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="n">
-        <v>60</v>
-      </c>
-      <c r="B62" t="n">
-        <v>102</v>
-      </c>
-      <c r="C62" t="n">
-        <v>24566</v>
+        <v>750</v>
       </c>
     </row>
   </sheetData>
@@ -2036,7 +1425,7 @@
         </is>
       </c>
       <c r="B2" s="5" t="n">
-        <v>92.01000000000001</v>
+        <v>11.93</v>
       </c>
     </row>
     <row r="3">
@@ -2046,7 +1435,7 @@
         </is>
       </c>
       <c r="B3" s="5" t="n">
-        <v>105.27</v>
+        <v>14.88</v>
       </c>
     </row>
     <row r="4">
@@ -2056,7 +1445,7 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>114.76</v>
+        <v>16.47</v>
       </c>
     </row>
     <row r="5">
@@ -2066,7 +1455,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>147.51</v>
+        <v>20.49</v>
       </c>
     </row>
     <row r="6">
@@ -2076,7 +1465,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>207.02</v>
+        <v>27.46</v>
       </c>
     </row>
     <row r="7">
@@ -2086,7 +1475,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>312.84</v>
+        <v>40.46</v>
       </c>
     </row>
     <row r="8">
@@ -2096,7 +1485,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>406.84</v>
+        <v>51.9</v>
       </c>
     </row>
     <row r="9">
@@ -2106,7 +1495,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>468.78</v>
+        <v>59.48</v>
       </c>
     </row>
     <row r="10">
@@ -2116,7 +1505,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>720.17</v>
+        <v>83.97</v>
       </c>
     </row>
     <row r="11">
@@ -2126,7 +1515,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>776.0599999999999</v>
+        <v>322.32</v>
       </c>
     </row>
     <row r="12">
@@ -2136,7 +1525,7 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>830.5599999999999</v>
+        <v>323.53</v>
       </c>
     </row>
     <row r="13">
@@ -2146,7 +1535,7 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>1052.27</v>
+        <v>323.53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>